<commit_message>
Actualizacao da analise dos indicadores
</commit_message>
<xml_diff>
--- a/Financeiro_Report.xlsx
+++ b/Financeiro_Report.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI13"/>
+  <dimension ref="A1:AI21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>350</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>350</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3918786000010380004</t>
+          <t>3918786000010395008</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -624,37 +624,37 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>3918786000010287026</t>
+          <t>3918786000010287028</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>3918786000010295044</t>
+          <t>3918786000010295056</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>GRACA CHICO PAULO VAGOS</t>
+          <t>LATIZA AIUBA</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>GRACA CHICO PAULO VAGOS</t>
+          <t>LATIZA AIUBA</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10900</t>
+          <t>33900</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>3135</t>
+          <t>500</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -721,17 +721,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>22900</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>7265</t>
+          <t>10500</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3918786000010380002</t>
+          <t>3918786000010395006</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -786,22 +786,22 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>3918786000010295062</t>
+          <t>3918786000010295018</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>MARAVILHA JANUARIO  CARIA</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>MARAVILHA JANUARIO  CARIA</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5480</t>
+          <t>36000</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3530</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -868,17 +868,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>600</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1680</t>
+          <t>35400</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>3918786000010379008</t>
+          <t>3918786000010395004</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>09-Jun-2026</t>
+          <t>08-Jun-2026</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>3918786000010295042</t>
+          <t>3918786000010295018</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -980,12 +980,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3750</t>
+          <t>1510</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1525</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1015,17 +1015,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3750</t>
+          <t>-235</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teve prejuízo na semana porque estava ocupada e nao conseguiu produzir </t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>3918786000010379006</t>
+          <t>3918786000010395002</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1050,7 +1055,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1065,37 +1070,37 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>3918786000010287028</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>3918786000010295056</t>
+          <t>3918786000010295042</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -1127,12 +1132,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10130</t>
+          <t>600</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2645</t>
+          <t>450</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1162,17 +1167,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>6885</t>
+          <t>90</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3918786000010379004</t>
+          <t>3918786000010390008</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1197,7 +1202,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1227,22 +1232,22 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>3918786000010295040</t>
+          <t>3918786000010295012</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>ASSINA ABDALA ABDULSATAR</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>ASSINA ABDALA ABDULSATAR</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1274,12 +1279,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>11750</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1160</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1309,17 +1314,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>490</t>
+          <t>470</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8410</t>
+          <t>10120</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>3918786000010379002</t>
+          <t>3918786000010390006</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1344,7 +1349,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1374,22 +1379,22 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>3918786000010295058</t>
+          <t>3918786000010295010</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -1416,17 +1421,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>17495</t>
+          <t>2180</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8960</t>
+          <t>1320</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1456,17 +1461,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4670</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3865</t>
+          <t>760</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>3918786000010367048</t>
+          <t>3918786000010390004</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1491,7 +1496,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1521,22 +1526,22 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>3918786000010295026</t>
+          <t>3918786000010295040</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>ELVIRA LOGRIGUES  MATANHA</t>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>ELVIRA LOGRIGUES  MATANHA</t>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1563,17 +1568,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9125</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1595</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1583,7 +1588,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1603,17 +1608,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>7430</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>3918786000010367046</t>
+          <t>3918786000010390002</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1633,17 +1638,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Investiu 160 na compra de formas novas</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1658,32 +1658,32 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>3918786000010295054</t>
+          <t>3918786000010295010</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>KHADYA AMADE SILIMO</t>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>KHADYA AMADE SILIMO</t>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
@@ -1715,57 +1715,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>3918786000004909039</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>550</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>3918786000010358004</t>
+          <t>3918786000010380004</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1788,14 +1788,9 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Trabalhar na visibilidade do negócio (fazer um plano de postagem)</t>
-        </is>
-      </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>09-Jun-2026</t>
+          <t>08-Jun-2026</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1810,32 +1805,32 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>3918786000010295012</t>
+          <t>3918786000010295044</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>GRACA CHICO PAULO VAGOS</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>GRACA CHICO PAULO VAGOS</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
@@ -1872,12 +1867,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18500</t>
+          <t>10900</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>5850</t>
+          <t>3135</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1907,17 +1902,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>500</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>11150</t>
+          <t>7265</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>3918786000010358002</t>
+          <t>3918786000010380002</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1972,17 +1967,17 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>3918786000010295052</t>
+          <t>3918786000010295062</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>JESSICA MARIA JOSE NAMUE</t>
+          <t>MARAVILHA JANUARIO  CARIA</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>JESSICA MARIA JOSE NAMUE</t>
+          <t>MARAVILHA JANUARIO  CARIA</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
@@ -2019,12 +2014,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1350</t>
+          <t>5480</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>3530</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2054,17 +2049,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>270</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>1680</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>3918786000010356002</t>
+          <t>3918786000010379008</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2089,7 +2084,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>09-Jun-2026</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -2104,32 +2099,32 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>3918786000010287028</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>3918786000010295090</t>
+          <t>3918786000010295042</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>TEODORA MANUEL BRAS</t>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>TEODORA MANUEL BRAS</t>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
@@ -2166,140 +2161,1326 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>3750</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>3750</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>3918786000010379006</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>3918786000010287028</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>3918786000010295056</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>LATIZA AIUBA</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>LATIZA AIUBA</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10130</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2645</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>6885</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>3918786000010379004</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>3918786000010295040</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>490</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>8410</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>3918786000010379002</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>3918786000010287026</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>3918786000010295058</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>17495</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>8960</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>4670</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3865</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>3918786000010367048</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>3918786000010295026</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>ELVIRA LOGRIGUES  MATANHA</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>ELVIRA LOGRIGUES  MATANHA</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>9125</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1595</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>7430</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>3918786000010367046</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Investiu 160 na compra de formas novas</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>3918786000010295054</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>KHADYA AMADE SILIMO</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>KHADYA AMADE SILIMO</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>3918786000010358004</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Trabalhar na visibilidade do negócio (fazer um plano de postagem)</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>09-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>3918786000010295012</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18500</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>5850</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>11150</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>3918786000010358002</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>3918786000010295052</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>JESSICA MARIA JOSE NAMUE</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>JESSICA MARIA JOSE NAMUE</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>3918786000010356002</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>3918786000010287028</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>3918786000010295090</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>TEODORA MANUEL BRAS</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>TEODORA MANUEL BRAS</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>13160</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>3705</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
         <is>
           <t>3918786000004909039</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>1005</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>8450</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>3918786000010353002</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>3918786000004909063</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>NAMPULA</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>NAMPULA</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
         <is>
           <t>08-Jun-2026</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>Luisa</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>Primeiro Mes de Implementação</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t>3918786000010287030</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AB21" t="inlineStr">
         <is>
           <t>3918786000010295028</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AC21" t="inlineStr">
         <is>
           <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
-      <c r="AD13" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
+      <c r="AE21" t="inlineStr">
         <is>
           <t>Primeira Semana</t>
         </is>
       </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr">
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
         <is>
           <t>3918786000007161003</t>
         </is>
       </c>
-      <c r="AI13" t="inlineStr">
+      <c r="AI21" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -2566,13 +3747,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD4CB22-937A-4AD3-8C0C-05205B420FA5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E11E11B-A02D-4B48-986F-BAB168800AF6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{690BED69-35F3-4FCA-9E13-D9C12FB24CD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B2D074-CB06-454B-80B6-5FDAAF6EB871}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55066A03-7AEC-4FA6-9D71-5E914A78F918}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CC285D4-43DE-4CBC-9F99-49DBE5D481C7}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao graficos de presencas por tipo sessao
</commit_message>
<xml_diff>
--- a/Financeiro_Report.xlsx
+++ b/Financeiro_Report.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI21"/>
+  <dimension ref="A1:AI37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>10800</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>620</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -574,17 +574,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>10080</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>3918786000010395008</t>
+          <t>3918786000010408006</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -604,12 +604,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -624,37 +624,37 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>3918786000010287028</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>3918786000010295056</t>
+          <t>3918786000010295036</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>FILOMENA AMINA DOMINGOS ALVEZ</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>FILOMENA AMINA DOMINGOS ALVEZ</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Segunda Semana</t>
+          <t>Primeira Semana</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33900</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -721,17 +721,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>22900</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10500</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3918786000010395006</t>
+          <t>3918786000010408004</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -771,32 +771,32 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>3918786000010295018</t>
+          <t>3918786000010295088</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>CATIZA ABAI NURO SITE</t>
+          <t>SUZANA JOAQUIM VAQUINA</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>CATIZA ABAI NURO SITE</t>
+          <t>SUZANA JOAQUIM VAQUINA</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>36000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -868,17 +868,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>35400</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>3918786000010395004</t>
+          <t>3918786000010408002</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -898,12 +898,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -918,32 +918,32 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>3918786000010295018</t>
+          <t>3918786000010295088</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>CATIZA ABAI NURO SITE</t>
+          <t>SUZANA JOAQUIM VAQUINA</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>CATIZA ABAI NURO SITE</t>
+          <t>SUZANA JOAQUIM VAQUINA</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
@@ -980,12 +980,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1510</t>
+          <t>6850</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1525</t>
+          <t>1320</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1015,22 +1015,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>600</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>-235</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">teve prejuízo na semana porque estava ocupada e nao conseguiu produzir </t>
+          <t>4930</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>3918786000010395002</t>
+          <t>3918786000010403026</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1055,7 +1050,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1085,17 +1080,17 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>3918786000010295042</t>
+          <t>3918786000010295052</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>JESSICA MARIA JOSE NAMUE</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>JESSICA MARIA JOSE NAMUE</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
@@ -1132,12 +1127,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>450</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1147,7 +1142,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1167,17 +1162,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3918786000010390008</t>
+          <t>3918786000010403024</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1202,7 +1197,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1217,32 +1212,32 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>3918786000010295012</t>
+          <t>3918786000010295044</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>GRACA CHICO PAULO VAGOS</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>GRACA CHICO PAULO VAGOS</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
@@ -1279,12 +1274,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11750</t>
+          <t>450</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1160</t>
+          <t>375</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1314,17 +1309,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>10120</t>
+          <t>75</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>3918786000010390006</t>
+          <t>3918786000010403022</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1349,7 +1344,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1379,17 +1374,17 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>3918786000010295010</t>
+          <t>3918786000010295090</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>ARISTINA RABIA JULIO MANUEL</t>
+          <t>TEODORA MANUEL BRAS</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>ARISTINA RABIA JULIO MANUEL</t>
+          <t>TEODORA MANUEL BRAS</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
@@ -1421,17 +1416,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2180</t>
+          <t>4800</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1320</t>
+          <t>835</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1461,17 +1456,17 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>760</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>3918786000010390004</t>
+          <t>3918786000010403020</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1496,7 +1491,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1526,17 +1521,17 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>3918786000010295040</t>
+          <t>3918786000010295062</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>MARAVILHA JANUARIO  CARIA</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>MARAVILHA JANUARIO  CARIA</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
@@ -1573,52 +1568,52 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>2955</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1220</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>3918786000004909039</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1735</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>3918786000010390002</t>
+          <t>3918786000010403018</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1638,12 +1633,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>15-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1658,37 +1653,37 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>3918786000010287026</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>3918786000010295010</t>
+          <t>3918786000010295054</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>ARISTINA RABIA JULIO MANUEL</t>
+          <t>KHADYA AMADE SILIMO</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>ARISTINA RABIA JULIO MANUEL</t>
+          <t>KHADYA AMADE SILIMO</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -1715,17 +1710,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>25175</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1880</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1735,7 +1730,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1755,17 +1750,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4470</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>18825</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>3918786000010380004</t>
+          <t>3918786000010403016</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1788,9 +1783,14 @@
           <t>Sim</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Investiu uma parte do lucro</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1805,37 +1805,37 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>3918786000010287026</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>3918786000010295044</t>
+          <t>3918786000010295036</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>GRACA CHICO PAULO VAGOS</t>
+          <t>FILOMENA AMINA DOMINGOS ALVEZ</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>GRACA CHICO PAULO VAGOS</t>
+          <t>FILOMENA AMINA DOMINGOS ALVEZ</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -1867,12 +1867,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10900</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3135</t>
+          <t>250</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1902,17 +1902,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>7265</t>
+          <t>850</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>3918786000010380002</t>
+          <t>3918786000010403014</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1952,37 +1952,37 @@
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>3918786000010295062</t>
+          <t>3918786000010295038</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>MARAVILHA JANUARIO  CARIA</t>
+          <t>FRANCISCA LUCIANO BOMES</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>MARAVILHA JANUARIO  CARIA</t>
+          <t>FRANCISCA LUCIANO BOMES</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -2014,12 +2014,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5480</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3530</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2049,17 +2049,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1680</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>3918786000010379008</t>
+          <t>3918786000010403012</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>09-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -2099,32 +2099,32 @@
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287026</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>3918786000010295042</t>
+          <t>3918786000010295038</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>FRANCISCA LUCIANO BOMES</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>GLORIA DA CONSTANCIA LOJA</t>
+          <t>FRANCISCA LUCIANO BOMES</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3750</t>
+          <t>3600</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2196,17 +2196,17 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>190</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3750</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>3918786000010379006</t>
+          <t>3918786000010403010</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -2246,32 +2246,32 @@
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>3918786000010287028</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>3918786000010295056</t>
+          <t>3918786000010295016</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>BENUA FERNANDO VALENTIM INACIO BENE</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>LATIZA AIUBA</t>
+          <t>BENUA FERNANDO VALENTIM INACIO BENE</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10130</t>
+          <t>5310</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2645</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2343,17 +2343,17 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>1320</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>6885</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>3918786000010379004</t>
+          <t>3918786000010403008</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -2408,22 +2408,22 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>3918786000010295040</t>
+          <t>3918786000010295016</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>BENUA FERNANDO VALENTIM INACIO BENE</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+          <t>BENUA FERNANDO VALENTIM INACIO BENE</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>9050</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>660</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2490,17 +2490,17 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>490</t>
+          <t>870</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>8410</t>
+          <t>7520</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>3918786000010379002</t>
+          <t>3918786000010403006</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -2602,12 +2602,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>17495</t>
+          <t>4985</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>8960</t>
+          <t>240</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2637,17 +2637,17 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>4670</t>
+          <t>520</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3865</t>
+          <t>4225</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>3918786000010367048</t>
+          <t>3918786000010403004</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -2744,17 +2744,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>9125</t>
+          <t>7600</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1595</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2784,17 +2784,17 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>5000</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>7430</t>
+          <t>1390</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>3918786000010367046</t>
+          <t>3918786000010403002</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2814,17 +2814,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Investiu 160 na compra de formas novas</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2854,22 +2849,22 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>3918786000010295054</t>
+          <t>3918786000010295028</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>KHADYA AMADE SILIMO</t>
+          <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>KHADYA AMADE SILIMO</t>
+          <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -2896,57 +2891,57 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>3918786000004909039</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>350</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>3918786000010358004</t>
+          <t>3918786000010395008</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2969,14 +2964,9 @@
           <t>Sim</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Trabalhar na visibilidade do negócio (fazer um plano de postagem)</t>
-        </is>
-      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>09-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2991,37 +2981,37 @@
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>3918786000010287030</t>
+          <t>3918786000010287028</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>3918786000010295012</t>
+          <t>3918786000010295056</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>LATIZA AIUBA</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>ASSINA ABDALA ABDULSATAR</t>
+          <t>LATIZA AIUBA</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -3053,12 +3043,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>18500</t>
+          <t>33900</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5850</t>
+          <t>500</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -3088,17 +3078,17 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>22900</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>11150</t>
+          <t>10500</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>3918786000010358002</t>
+          <t>3918786000010395006</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -3123,7 +3113,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>08-Jun-2026</t>
+          <t>15-Jun-2026</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -3153,22 +3143,22 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>3918786000010295052</t>
+          <t>3918786000010295018</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>JESSICA MARIA JOSE NAMUE</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>JESSICA MARIA JOSE NAMUE</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>Primeira Semana</t>
+          <t>Segunda Semana</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -3200,12 +3190,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1350</t>
+          <t>36000</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>930</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -3235,17 +3225,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>600</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>35400</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>3918786000010356002</t>
+          <t>3918786000010395004</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -3285,32 +3275,32 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>3918786000010287028</t>
+          <t>3918786000010287030</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>3918786000010295090</t>
+          <t>3918786000010295018</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>TEODORA MANUEL BRAS</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>TEODORA MANUEL BRAS</t>
+          <t>CATIZA ABAI NURO SITE</t>
         </is>
       </c>
       <c r="AE20" t="inlineStr">
@@ -3347,140 +3337,2507 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1525</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>-235</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">teve prejuízo na semana porque estava ocupada e nao conseguiu produzir </t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>3918786000010395002</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>15-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>3918786000010295042</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>Segunda Semana</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>3918786000010390008</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>15-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>3918786000010295012</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>Segunda Semana</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11750</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1160</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>10120</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>3918786000010390006</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>15-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>3918786000010287026</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>3918786000010295010</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>Segunda Semana</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2180</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1320</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>760</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>3918786000010390004</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>15-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>3918786000010295040</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>Segunda Semana</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>3918786000010390002</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>15-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>3918786000010287026</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>3918786000010295010</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>ARISTINA RABIA JULIO MANUEL</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>3918786000010380004</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>3918786000010287026</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>3918786000010295044</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>GRACA CHICO PAULO VAGOS</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>GRACA CHICO PAULO VAGOS</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10900</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>3135</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>7265</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>3918786000010380002</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>3918786000010295062</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>MARAVILHA JANUARIO  CARIA</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>MARAVILHA JANUARIO  CARIA</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>5480</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>3530</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1680</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>3918786000010379008</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>09-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>3918786000010295042</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>GLORIA DA CONSTANCIA LOJA</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3750</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3750</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>3918786000010379006</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>3918786000010287028</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>3918786000010295056</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>LATIZA AIUBA</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>LATIZA AIUBA</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10130</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2645</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>600</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>6885</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>3918786000010379004</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>3918786000010295040</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>GLORIA  GERMANO DO ROSARIO RIBEIRO</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>490</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>8410</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>3918786000010379002</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>3918786000010287026</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Prestação de serviços (ornamentação de eventos, microcrédito, salão de cabeleleiro, takeaway etc)</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>3918786000010295058</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>LUCIA  EUGENIO LUCIANO VIEGAS</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17495</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8960</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>4670</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>3865</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>3918786000010367048</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>3918786000010295026</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>ELVIRA LOGRIGUES  MATANHA</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>ELVIRA LOGRIGUES  MATANHA</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>9125</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1595</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>7430</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>3918786000010367046</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Investiu 160 na compra de formas novas</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>3918786000010295054</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>KHADYA AMADE SILIMO</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>KHADYA AMADE SILIMO</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>3918786000010358004</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Trabalhar na visibilidade do negócio (fazer um plano de postagem)</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>09-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>3918786000010295012</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>ASSINA ABDALA ABDULSATAR</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18500</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5850</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>11150</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>3918786000010358002</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>3918786000010287030</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>3918786000010295052</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>JESSICA MARIA JOSE NAMUE</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>JESSICA MARIA JOSE NAMUE</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1350</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>930</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>3918786000004909039</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>3918786000010356002</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>3918786000004909063</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>08-Jun-2026</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Luisa</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Primeiro Mes de Implementação</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>3918786000010287028</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Produção e venda de produtos não alimentares (Artesanato, etc: Com transformação de prod.)</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>3918786000010295090</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>TEODORA MANUEL BRAS</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>TEODORA MANUEL BRAS</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>Primeira Semana</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>3918786000007161003</t>
+        </is>
+      </c>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>13160</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>3705</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>3918786000004909039</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>PAM VERDE</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>PAM VERDE</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>1005</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>8450</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>3918786000010353002</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>3918786000004909063</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>NAMPULA</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>NAMPULA</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr">
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>NAMPULA</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
         <is>
           <t>08-Jun-2026</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>Luisa</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="W37" t="inlineStr">
         <is>
           <t>Primeiro Mes de Implementação</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="Y37" t="inlineStr">
         <is>
           <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="Z37" t="inlineStr">
         <is>
           <t>3918786000010287030</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AA37" t="inlineStr">
         <is>
           <t>Produção e venda de produtos alimentares (bolos, salgados, comidas, etc :transformação de prod)</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AB37" t="inlineStr">
         <is>
           <t>3918786000010295028</t>
         </is>
       </c>
-      <c r="AC21" t="inlineStr">
+      <c r="AC37" t="inlineStr">
         <is>
           <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
-      <c r="AD21" t="inlineStr">
+      <c r="AD37" t="inlineStr">
         <is>
           <t>ESMERALDA JORGE MURIRIUA</t>
         </is>
       </c>
-      <c r="AE21" t="inlineStr">
+      <c r="AE37" t="inlineStr">
         <is>
           <t>Primeira Semana</t>
         </is>
       </c>
-      <c r="AF21" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="AH21" t="inlineStr">
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
         <is>
           <t>3918786000007161003</t>
         </is>
       </c>
-      <c r="AI21" t="inlineStr">
+      <c r="AI37" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
@@ -3747,13 +6104,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E11E11B-A02D-4B48-986F-BAB168800AF6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2669AFD-A6A7-4513-90EA-B57CCB675D35}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B2D074-CB06-454B-80B6-5FDAAF6EB871}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02D3D0F8-03FD-456A-9CB8-EBDE37C5E645}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CC285D4-43DE-4CBC-9F99-49DBE5D481C7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51819B3A-A689-49E9-A39D-1118DCA4C2E1}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao da pagina Beira
</commit_message>
<xml_diff>
--- a/Financeiro_Report.xlsx
+++ b/Financeiro_Report.xlsx
@@ -31733,13 +31733,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6398845F-9212-4610-BE7D-65CDE4D29B07}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BF5AE61-9896-43D2-9BD5-772FC45D03EC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C4C49C-6AEB-4A4A-8BF5-1739F7E1F8F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBB82439-B654-4221-B0FF-BE574EC74CF0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6AA6967F-CCFB-44C1-9BD6-E3CC19A81CE1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A2C4497-03F6-41DA-AEE1-E888C052840E}"/>
 </file>
</xml_diff>